<commit_message>
boundary value analysis - FR-03
</commit_message>
<xml_diff>
--- a/reports/FR-03_domain_test_cases.xlsx
+++ b/reports/FR-03_domain_test_cases.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="195">
   <si>
     <t>Giả định và câu hỏi mở</t>
   </si>
@@ -548,33 +548,12 @@
     <t>Accepted; mật khẩu được đổi thành công.</t>
   </si>
   <si>
-    <t>Không thể thực hiện test vì chương trình sinh mã OTP 4 chữ số (lỗi ER-FR03-01).</t>
-  </si>
-  <si>
     <t>ER-FR03-02</t>
   </si>
   <si>
-    <t>New Pass12</t>
-  </si>
-  <si>
     <t>Rejected; yêu cầu nhập mật khẩu mới</t>
   </si>
   <si>
-    <t>New Pass!!</t>
-  </si>
-  <si>
-    <t>NEW PASS1!</t>
-  </si>
-  <si>
-    <t>new pass1!</t>
-  </si>
-  <si>
-    <t>New Pass1#!</t>
-  </si>
-  <si>
-    <t>Không thể thực hiện test vì giao diện không có trường xác nhận mật khẩu mới (lỗi UI)</t>
-  </si>
-  <si>
     <t>Không có chỉ báo số bước</t>
   </si>
   <si>
@@ -590,20 +569,60 @@
     <t>Rejected; OTP không đúng</t>
   </si>
   <si>
-    <t>Aa !1yz</t>
-  </si>
-  <si>
-    <t>Hệ thống không áp dụng thời hạn OTP</t>
-  </si>
-  <si>
     <t>Ghi chú</t>
+  </si>
+  <si>
+    <t>ER-FR03-04</t>
+  </si>
+  <si>
+    <t>Không có trường Xác nhận mật khẩu mới</t>
+  </si>
+  <si>
+    <t>Không thể thực hiện test vì giao diện không có trường xác nhận mật khẩu mới (ER-FR03-04)</t>
+  </si>
+  <si>
+    <t>Đặc tả không ghi rõ thời hạn OTP để thực hiện test.</t>
+  </si>
+  <si>
+    <t>TC-FR03-38</t>
+  </si>
+  <si>
+    <t>Bảng test cases sử dụng giá trị minh họa, thay bằng giá trị thực tế khi test.
+-&gt; Không thể thực hiện test vì chương trình sinh mã OTP 4 chữ số (lỗi ER-FR03-01).</t>
+  </si>
+  <si>
+    <t>Không khớp với OTP đã tạo cho tài khoản</t>
+  </si>
+  <si>
+    <t>582731 (giá trị hệ thống tạo là 482731)</t>
+  </si>
+  <si>
+    <t>Rejected; OTP không đúng.</t>
+  </si>
+  <si>
+    <t>Aab!1yz</t>
+  </si>
+  <si>
+    <t>NewPass1#</t>
+  </si>
+  <si>
+    <t>NewPass12</t>
+  </si>
+  <si>
+    <t>NewPass!!</t>
+  </si>
+  <si>
+    <t>NEWPASS1!</t>
+  </si>
+  <si>
+    <t>newpass1!</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -621,14 +640,6 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -660,7 +671,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -680,7 +691,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1198,7 +1212,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" style="3" customWidth="1"/>
@@ -1239,7 +1253,7 @@
         <v>120</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -1383,7 +1397,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>128</v>
       </c>
@@ -1403,10 +1417,10 @@
         <v>161</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>129</v>
       </c>
@@ -1427,7 +1441,7 @@
       </c>
       <c r="I9" s="7"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>130</v>
       </c>
@@ -1580,7 +1594,7 @@
         <v>72</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>160</v>
@@ -1606,7 +1620,7 @@
         <v>168</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
@@ -1626,7 +1640,7 @@
         <v>78</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>160</v>
@@ -1648,14 +1662,14 @@
       <c r="E19" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="F19" s="6" t="s">
         <v>83</v>
       </c>
       <c r="G19" s="3" t="s">
         <v>121</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -1675,7 +1689,7 @@
         <v>50</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="G20" s="3" t="s">
         <v>160</v>
@@ -1721,7 +1735,7 @@
         <v>57</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="G22" s="3" t="s">
         <v>160</v>
@@ -1738,7 +1752,7 @@
         <v>84</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>178</v>
+        <v>194</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>83</v>
@@ -1762,7 +1776,7 @@
         <v>85</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>177</v>
+        <v>193</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>83</v>
@@ -1786,7 +1800,7 @@
         <v>86</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>83</v>
@@ -1810,19 +1824,16 @@
         <v>87</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>174</v>
+        <v>191</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>83</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>171</v>
+        <v>83</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="H26" s="3" t="s">
-        <v>173</v>
+        <v>160</v>
       </c>
       <c r="I26" s="2"/>
     </row>
@@ -1837,7 +1848,7 @@
         <v>88</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>89</v>
@@ -1848,6 +1859,7 @@
       <c r="G27" s="3" t="s">
         <v>160</v>
       </c>
+      <c r="H27" s="6"/>
       <c r="I27" s="2"/>
     </row>
     <row r="28" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -1861,7 +1873,7 @@
         <v>90</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>91</v>
@@ -1874,7 +1886,7 @@
       </c>
       <c r="I28" s="2"/>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
         <v>149</v>
       </c>
@@ -1890,14 +1902,17 @@
       <c r="E29" s="3" t="s">
         <v>94</v>
       </c>
+      <c r="F29" s="3" t="s">
+        <v>181</v>
+      </c>
       <c r="G29" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="I29" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="H29" s="3" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>150</v>
       </c>
@@ -1916,7 +1931,9 @@
       <c r="G30" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="I30" s="6"/>
+      <c r="I30" s="8" t="s">
+        <v>182</v>
+      </c>
     </row>
     <row r="31" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
@@ -1937,7 +1954,7 @@
       <c r="G31" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="I31" s="6"/>
+      <c r="I31" s="8"/>
     </row>
     <row r="32" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
@@ -1958,7 +1975,7 @@
       <c r="G32" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="I32" s="6"/>
+      <c r="I32" s="8"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
@@ -1979,7 +1996,7 @@
       <c r="G33" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="I33" s="6"/>
+      <c r="I33" s="8"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
@@ -1998,13 +2015,13 @@
         <v>102</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="G34" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="H34" s="6" t="s">
-        <v>182</v>
+      <c r="H34" s="8" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
@@ -2024,12 +2041,12 @@
         <v>102</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="G35" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="H35" s="6"/>
+      <c r="H35" s="8"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
@@ -2048,12 +2065,12 @@
         <v>107</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="G36" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="H36" s="6"/>
+      <c r="H36" s="8"/>
     </row>
     <row r="37" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
@@ -2072,12 +2089,12 @@
         <v>110</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="H37" s="6"/>
+      <c r="H37" s="8"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
@@ -2096,18 +2113,47 @@
         <v>113</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="G38" s="3" t="s">
         <v>161</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A39" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="I39" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A40" s="6"/>
+      <c r="B40" s="6" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E38"/>
   <mergeCells count="3">
     <mergeCell ref="I8:I10"/>
-    <mergeCell ref="I29:I33"/>
     <mergeCell ref="H34:H37"/>
+    <mergeCell ref="I30:I33"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D3" r:id="rId1"/>

</xml_diff>